<commit_message>
PCF-0: address review (leg mass, placeholder banners, cut-off and primary-data rules)
- transport legs carry mass_t_per_unit; method note says it maps to E1 payload_t
- red placeholder banner and tab on every sheet
- per-line cut_off_candidate in expected.lines; A3 energy lines excluded, stated in the note
- primary data defined by activity data; flagged for sign-off
- allocation lines renamed A3E1-A3E4; reconciliation note on single-product coverage

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014zs279WstN2feG4U4wCMoZ
</commit_message>
<xml_diff>
--- a/docs/pcf/phase0/pilot-golden.xlsx
+++ b/docs/pcf/phase0/pilot-golden.xlsx
@@ -542,14 +542,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00B00020"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -563,6 +565,12 @@
           <t>Value</t>
         </is>
       </c>
+      <c r="C1" s="3" t="n"/>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER NUMBERS · not Midal data</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -575,6 +583,8 @@
           <t>EC-grade aluminium wire rod 9.5 mm</t>
         </is>
       </c>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -587,6 +597,8 @@
           <t>Midal Cables (pilot)</t>
         </is>
       </c>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -599,6 +611,8 @@
           <t>Bahrain plant (placeholder)</t>
         </is>
       </c>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -611,6 +625,8 @@
           <t>kg</t>
         </is>
       </c>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -621,6 +637,8 @@
       <c r="B6" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -631,6 +649,8 @@
       <c r="B7" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -643,6 +663,8 @@
           <t>2025-01-01</t>
         </is>
       </c>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -655,6 +677,8 @@
           <t>2025-12-31</t>
         </is>
       </c>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -667,6 +691,8 @@
           <t>CY</t>
         </is>
       </c>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -679,6 +705,8 @@
           <t>cradle_to_gate</t>
         </is>
       </c>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -691,6 +719,8 @@
           <t>iso14067</t>
         </is>
       </c>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -703,6 +733,8 @@
           <t>PEP PCR-ed4 / EN 50693 (optional)</t>
         </is>
       </c>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -715,6 +747,8 @@
           <t>mass</t>
         </is>
       </c>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -725,6 +759,8 @@
       <c r="B15" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -735,6 +771,8 @@
       <c r="B16" s="5" t="n">
         <v>5</v>
       </c>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -747,6 +785,8 @@
           <t>AR6</t>
         </is>
       </c>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -756,10 +796,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00B00020"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -770,6 +811,7 @@
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="58" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -813,6 +855,12 @@
           <t>licence</t>
         </is>
       </c>
+      <c r="I1" s="3" t="n"/>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER NUMBERS · not Midal data</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -853,6 +901,8 @@
           <t>open</t>
         </is>
       </c>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -893,6 +943,8 @@
           <t>open</t>
         </is>
       </c>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -933,6 +985,8 @@
           <t>open</t>
         </is>
       </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -973,6 +1027,8 @@
           <t>open</t>
         </is>
       </c>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1013,6 +1069,8 @@
           <t>open</t>
         </is>
       </c>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1053,6 +1111,8 @@
           <t>open</t>
         </is>
       </c>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1093,6 +1153,8 @@
           <t>open</t>
         </is>
       </c>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1133,6 +1195,8 @@
           <t>open</t>
         </is>
       </c>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1173,6 +1237,8 @@
           <t>open</t>
         </is>
       </c>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1213,6 +1279,8 @@
           <t>open</t>
         </is>
       </c>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1253,6 +1321,8 @@
           <t>open</t>
         </is>
       </c>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1262,10 +1332,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00B00020"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1283,6 +1354,7 @@
     <col width="9" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1361,6 +1433,12 @@
           <t>dqr_time</t>
         </is>
       </c>
+      <c r="P1" s="3" t="n"/>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER NUMBERS · not Midal data</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1425,6 +1503,8 @@
       <c r="O2" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="P2" s="3" t="n"/>
+      <c r="Q2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1485,6 +1565,8 @@
       <c r="O3" s="5" t="n">
         <v>2</v>
       </c>
+      <c r="P3" s="3" t="n"/>
+      <c r="Q3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1545,6 +1627,8 @@
       <c r="O4" s="5" t="n">
         <v>2</v>
       </c>
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1605,6 +1689,8 @@
       <c r="O5" s="5" t="n">
         <v>2</v>
       </c>
+      <c r="P5" s="3" t="n"/>
+      <c r="Q5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1665,6 +1751,8 @@
       <c r="O6" s="5" t="n">
         <v>2</v>
       </c>
+      <c r="P6" s="3" t="n"/>
+      <c r="Q6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1725,6 +1813,8 @@
       <c r="O7" s="5" t="n">
         <v>2</v>
       </c>
+      <c r="P7" s="3" t="n"/>
+      <c r="Q7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1785,6 +1875,8 @@
       <c r="O8" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="P8" s="3" t="n"/>
+      <c r="Q8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1845,6 +1937,8 @@
       <c r="O9" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="P9" s="3" t="n"/>
+      <c r="Q9" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1854,10 +1948,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00B00020"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1873,6 +1968,7 @@
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="9" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1941,6 +2037,12 @@
           <t>dqr_time</t>
         </is>
       </c>
+      <c r="N1" s="3" t="n"/>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER NUMBERS · not Midal data</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1997,6 +2099,8 @@
       <c r="M2" s="5" t="n">
         <v>1</v>
       </c>
+      <c r="N2" s="3" t="n"/>
+      <c r="O2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -2053,6 +2157,8 @@
       <c r="M3" s="5" t="n">
         <v>2</v>
       </c>
+      <c r="N3" s="3" t="n"/>
+      <c r="O3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2109,6 +2215,8 @@
       <c r="M4" s="5" t="n">
         <v>2</v>
       </c>
+      <c r="N4" s="3" t="n"/>
+      <c r="O4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2165,6 +2273,8 @@
       <c r="M5" s="5" t="n">
         <v>2</v>
       </c>
+      <c r="N5" s="3" t="n"/>
+      <c r="O5" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2174,10 +2284,11 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00B00020"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2190,12 +2301,13 @@
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Approved ProductionData at the site in the reference period (t)</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Approved ProductionData at the site in the reference period (t) · PLACEHOLDER, not Midal data</t>
         </is>
       </c>
       <c r="B1" s="3" t="n"/>
@@ -2207,6 +2319,12 @@
       <c r="H1" s="3" t="n"/>
       <c r="I1" s="3" t="n"/>
       <c r="J1" s="3" t="n"/>
+      <c r="K1" s="3" t="n"/>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER NUMBERS · not Midal data</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -2227,6 +2345,8 @@
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -2245,6 +2365,8 @@
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2263,6 +2385,8 @@
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2281,6 +2405,8 @@
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2299,6 +2425,8 @@
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -2318,6 +2446,8 @@
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -2337,6 +2467,8 @@
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -2356,6 +2488,8 @@
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -2375,6 +2509,8 @@
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -2391,6 +2527,8 @@
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -2443,11 +2581,13 @@
           <t>dqr_time</t>
         </is>
       </c>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>A3E1</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2483,11 +2623,13 @@
       <c r="J13" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>A3E2</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2523,11 +2665,13 @@
       <c r="J14" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>A3E3</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2563,11 +2707,13 @@
       <c r="J15" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>A3E4</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2603,6 +2749,8 @@
       <c r="J16" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2612,10 +2760,11 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00B00020"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2628,6 +2777,7 @@
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2645,6 +2795,12 @@
       <c r="H1" s="3" t="n"/>
       <c r="I1" s="3" t="n"/>
       <c r="J1" s="3" t="n"/>
+      <c r="K1" s="3" t="n"/>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER NUMBERS · not Midal data</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n"/>
@@ -2657,6 +2813,8 @@
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -2709,6 +2867,8 @@
           <t>dqr_time</t>
         </is>
       </c>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3">
@@ -2751,6 +2911,8 @@
         <f>Inputs!O2</f>
         <v/>
       </c>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3">
@@ -2793,6 +2955,8 @@
         <f>Inputs!O3</f>
         <v/>
       </c>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3">
@@ -2835,6 +2999,8 @@
         <f>Inputs!O4</f>
         <v/>
       </c>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3">
@@ -2877,6 +3043,8 @@
         <f>Inputs!O5</f>
         <v/>
       </c>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3">
@@ -2919,6 +3087,8 @@
         <f>Inputs!O6</f>
         <v/>
       </c>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3">
@@ -2961,6 +3131,8 @@
         <f>Inputs!O7</f>
         <v/>
       </c>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3">
@@ -3003,6 +3175,8 @@
         <f>Inputs!O8</f>
         <v/>
       </c>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3">
@@ -3045,6 +3219,8 @@
         <f>Inputs!O9</f>
         <v/>
       </c>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3">
@@ -3087,6 +3263,8 @@
         <f>Transport!M2</f>
         <v/>
       </c>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3">
@@ -3129,6 +3307,8 @@
         <f>Transport!M3</f>
         <v/>
       </c>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3">
@@ -3171,6 +3351,8 @@
         <f>Transport!M4</f>
         <v/>
       </c>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3">
@@ -3213,6 +3395,8 @@
         <f>Transport!M5</f>
         <v/>
       </c>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3">
@@ -3257,6 +3441,8 @@
         <f>Allocation!J13</f>
         <v/>
       </c>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3">
@@ -3301,6 +3487,8 @@
         <f>Allocation!J14</f>
         <v/>
       </c>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3">
@@ -3345,6 +3533,8 @@
         <f>Allocation!J15</f>
         <v/>
       </c>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3">
@@ -3389,6 +3579,8 @@
         <f>Allocation!J16</f>
         <v/>
       </c>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -3401,6 +3593,8 @@
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
+      <c r="K20" s="3" t="n"/>
+      <c r="L20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -3417,6 +3611,8 @@
       <c r="H21" s="3" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
+      <c r="K21" s="3" t="n"/>
+      <c r="L21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -3436,6 +3632,8 @@
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -3455,6 +3653,8 @@
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -3474,6 +3674,8 @@
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="n"/>
+      <c r="L24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -3493,6 +3695,8 @@
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -3512,6 +3716,8 @@
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+      <c r="L26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -3531,6 +3737,8 @@
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
+      <c r="L27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -3543,6 +3751,8 @@
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
+      <c r="L28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -3562,6 +3772,8 @@
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
+      <c r="K29" s="3" t="n"/>
+      <c r="L29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -3581,6 +3793,8 @@
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
+      <c r="L30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -3600,6 +3814,8 @@
       <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
+      <c r="K31" s="3" t="n"/>
+      <c r="L31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -3619,6 +3835,8 @@
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
+      <c r="K32" s="3" t="n"/>
+      <c r="L32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -3638,6 +3856,8 @@
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
+      <c r="K33" s="3" t="n"/>
+      <c r="L33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -3650,6 +3870,8 @@
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
+      <c r="K34" s="3" t="n"/>
+      <c r="L34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -3669,6 +3891,8 @@
       <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
+      <c r="L35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -3688,6 +3912,8 @@
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
+      <c r="K36" s="3" t="n"/>
+      <c r="L36" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3697,27 +3923,37 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00B00020"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="66" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Σ PCF(A3 energy) × approved production vs plant Scope 1+2 (only the pilot is footprinted, so coverage is low by design)</t>
+          <t>Σ PCF(A3 energy) × approved production vs plant Scope 1+2 (only the pilot is footprinted, so coverage equals its allocation share by construction)</t>
         </is>
       </c>
       <c r="B1" s="3" t="n"/>
+      <c r="C1" s="3" t="n"/>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER NUMBERS · not Midal data</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n"/>
       <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -3729,6 +3965,8 @@
         <f>SUM(Allocation!D13:D16)</f>
         <v/>
       </c>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -3740,6 +3978,8 @@
         <f>Result!$D$25</f>
         <v/>
       </c>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -3751,6 +3991,8 @@
         <f>Allocation!$B$10</f>
         <v/>
       </c>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -3762,6 +4004,8 @@
         <f>B4*B5/1000</f>
         <v/>
       </c>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -3773,6 +4017,8 @@
         <f>B6/B3*100</f>
         <v/>
       </c>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -3784,6 +4030,8 @@
         <f>IF(B7&lt;90,"below 90%","ok")</f>
         <v/>
       </c>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>